<commit_message>
Compute real Embodied Carbon A1-A3 totals for area/length/count rows (B2)
Previously mass, and therefore A1-A3, was only derived for volume/weight
rows -- 35 area/length/count rows had Density/GWP populated but no total,
despite the README claiming full coverage. Most of those rows' BoQ
descriptions state an explicit thickness, cross-section, or per-unit rate
(e.g. '40 mm thick', '1.7 Kg. per square metre'), so parse those into
AREA_TO_MASS/LENGTH_TO_MASS/COUNT_TO_MASS lookups and derive mass from
them. Coverage goes from 16/51 to 35/51 rows with a computed total; the
rest (mostly count-based ironmongery with no stated per-unit mass) are
left blank rather than guessed. Also add a dedicated glass carbon entry
so item 43 ('Glass strips (terrazzo joints)') doesn't fall through to
the terrazzo/marble keyword match on the word 'terrazzo' in its label.
</commit_message>
<xml_diff>
--- a/output/passport_filled.xlsx
+++ b/output/passport_filled.xlsx
@@ -2115,7 +2115,9 @@
       <c r="X15" s="8" t="n">
         <v>2400</v>
       </c>
-      <c r="Y15" s="8" t="n"/>
+      <c r="Y15" s="8" t="n">
+        <v>179.7</v>
+      </c>
       <c r="Z15" s="8" t="n">
         <v>0.13</v>
       </c>
@@ -2156,7 +2158,7 @@
       </c>
       <c r="AX15" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - concrete, 30-35 MPa, general mix</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - concrete, 30-35 MPa, general mix; Mass derived from area x 40mm thickness (from BoQ description) x density</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2233,9 @@
       <c r="X16" s="8" t="n">
         <v>1050</v>
       </c>
-      <c r="Y16" s="8" t="n"/>
+      <c r="Y16" s="8" t="n">
+        <v>9.300000000000001</v>
+      </c>
       <c r="Z16" s="8" t="n">
         <v>0.38</v>
       </c>
@@ -2272,7 +2276,7 @@
       </c>
       <c r="AX16" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - bitumen</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - bitumen; Mass derived from DSR-stated coating rate 1.7 kg/sq.m</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4163,9 @@
       <c r="X32" s="8" t="n">
         <v>1800</v>
       </c>
-      <c r="Y32" s="8" t="n"/>
+      <c r="Y32" s="8" t="n">
+        <v>27.2</v>
+      </c>
       <c r="Z32" s="8" t="n">
         <v>0.24</v>
       </c>
@@ -4200,7 +4206,7 @@
       </c>
       <c r="AX32" s="8" t="inlineStr">
         <is>
-          <t>Brick class designation left blank in source BoQ per footnote ('appropriate class designation of bricks may be incorporated before calling tenders') - not a scan defect; Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - brick, common fired clay</t>
+          <t>Brick class designation left blank in source BoQ per footnote ('appropriate class designation of bricks may be incorporated before calling tenders') - not a scan defect; Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - brick, common fired clay; Mass derived from area x 70mm thickness (from BoQ description) x density</t>
         </is>
       </c>
     </row>
@@ -4283,7 +4289,9 @@
       <c r="X33" s="8" t="n">
         <v>1800</v>
       </c>
-      <c r="Y33" s="8" t="n"/>
+      <c r="Y33" s="8" t="n">
+        <v>238.5</v>
+      </c>
       <c r="Z33" s="8" t="n">
         <v>0.24</v>
       </c>
@@ -4324,7 +4332,7 @@
       </c>
       <c r="AX33" s="8" t="inlineStr">
         <is>
-          <t>Brick class designation left blank in source BoQ per footnote ('appropriate class designation of bricks may be incorporated before calling tenders') - not a scan defect; Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - brick, common fired clay</t>
+          <t>Brick class designation left blank in source BoQ per footnote ('appropriate class designation of bricks may be incorporated before calling tenders') - not a scan defect; Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - brick, common fired clay; Mass derived from area x 115mm thickness (from BoQ description) x density; Half-brick thickness assumed at standard 115mm nominal (not stated on scan)</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4415,9 @@
       <c r="X34" s="8" t="n">
         <v>1800</v>
       </c>
-      <c r="Y34" s="8" t="n"/>
+      <c r="Y34" s="8" t="n">
+        <v>894.2</v>
+      </c>
       <c r="Z34" s="8" t="n">
         <v>0.24</v>
       </c>
@@ -4448,7 +4458,7 @@
       </c>
       <c r="AX34" s="8" t="inlineStr">
         <is>
-          <t>Brick class designation left blank in source BoQ per footnote ('appropriate class designation of bricks may be incorporated before calling tenders') - not a scan defect; Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - brick, common fired clay</t>
+          <t>Brick class designation left blank in source BoQ per footnote ('appropriate class designation of bricks may be incorporated before calling tenders') - not a scan defect; Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - brick, common fired clay; Mass derived from area x 115mm thickness (from BoQ description) x density; Half-brick thickness assumed at standard 115mm nominal (not stated on scan)</t>
         </is>
       </c>
     </row>
@@ -4647,7 +4657,9 @@
       <c r="X36" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="Y36" s="8" t="n"/>
+      <c r="Y36" s="8" t="n">
+        <v>158.8</v>
+      </c>
       <c r="Z36" s="8" t="n">
         <v>0.42</v>
       </c>
@@ -4684,7 +4696,7 @@
       </c>
       <c r="AX36" s="8" t="inlineStr">
         <is>
-          <t>Wood species left blank in source BoQ per the same footnote; Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - timber, general hardwood sawn</t>
+          <t>Wood species left blank in source BoQ per the same footnote; Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - timber, general hardwood sawn; Mass derived from area x 35mm thickness (from BoQ description) x density</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4771,9 @@
       <c r="X37" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="Y37" s="8" t="n"/>
+      <c r="Y37" s="8" t="n">
+        <v>29.6</v>
+      </c>
       <c r="Z37" s="8" t="n">
         <v>0.42</v>
       </c>
@@ -4800,7 +4814,7 @@
       </c>
       <c r="AX37" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - timber, general hardwood sawn</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - timber, general hardwood sawn; Mass derived from area x 25mm thickness (from BoQ description) x density</t>
         </is>
       </c>
     </row>
@@ -6731,7 +6745,9 @@
       <c r="X54" s="8" t="n">
         <v>2400</v>
       </c>
-      <c r="Y54" s="8" t="n"/>
+      <c r="Y54" s="8" t="n">
+        <v>848.6</v>
+      </c>
       <c r="Z54" s="8" t="n">
         <v>0.13</v>
       </c>
@@ -6772,7 +6788,7 @@
       </c>
       <c r="AX54" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - concrete, 30-35 MPa, general mix</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - concrete, 30-35 MPa, general mix; Mass derived from area x 40mm thickness (from BoQ description) x density</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6871,9 @@
       <c r="X55" s="8" t="n">
         <v>1900</v>
       </c>
-      <c r="Y55" s="8" t="n"/>
+      <c r="Y55" s="8" t="n">
+        <v>59.1</v>
+      </c>
       <c r="Z55" s="8" t="n">
         <v>0.157</v>
       </c>
@@ -6896,7 +6914,7 @@
       </c>
       <c r="AX55" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - mortar (1:6 cement:sand, general)</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - mortar (1:6 cement:sand, general); Mass derived from area x 18mm thickness (from BoQ description) x density</t>
         </is>
       </c>
     </row>
@@ -6979,7 +6997,9 @@
       <c r="X56" s="8" t="n">
         <v>2700</v>
       </c>
-      <c r="Y56" s="8" t="n"/>
+      <c r="Y56" s="8" t="n">
+        <v>76.8</v>
+      </c>
       <c r="Z56" s="8" t="n">
         <v>0.079</v>
       </c>
@@ -7020,7 +7040,7 @@
       </c>
       <c r="AX56" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - marble/dimension stone</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - marble/dimension stone; Mass derived from area x 40mm thickness (from BoQ description) x density; Composite assembly: mass uses only the top finish layer's stated thickness/density; underlayer(s) of a different material are excluded</t>
         </is>
       </c>
     </row>
@@ -7093,11 +7113,13 @@
       <c r="V57" s="8" t="inlineStr"/>
       <c r="W57" s="8" t="inlineStr"/>
       <c r="X57" s="8" t="n">
-        <v>2700</v>
-      </c>
-      <c r="Y57" s="8" t="n"/>
+        <v>2500</v>
+      </c>
+      <c r="Y57" s="8" t="n">
+        <v>9.199999999999999</v>
+      </c>
       <c r="Z57" s="8" t="n">
-        <v>0.079</v>
+        <v>0.85</v>
       </c>
       <c r="AA57" s="8" t="inlineStr">
         <is>
@@ -7136,7 +7158,7 @@
       </c>
       <c r="AX57" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - marble/dimension stone</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - glass, general; Mass derived from length x 240.0 sq.mm cross-section (from BoQ description) x density</t>
         </is>
       </c>
     </row>
@@ -7211,7 +7233,9 @@
       <c r="X58" s="8" t="n">
         <v>1050</v>
       </c>
-      <c r="Y58" s="8" t="n"/>
+      <c r="Y58" s="8" t="n">
+        <v>42</v>
+      </c>
       <c r="Z58" s="8" t="n">
         <v>0.38</v>
       </c>
@@ -7252,7 +7276,7 @@
       </c>
       <c r="AX58" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - bitumen</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - bitumen; Mass derived from DSR-stated coating rate 1.7 kg/sq.m</t>
         </is>
       </c>
     </row>
@@ -7571,7 +7595,9 @@
       <c r="X61" s="8" t="n">
         <v>2400</v>
       </c>
-      <c r="Y61" s="8" t="n"/>
+      <c r="Y61" s="8" t="n">
+        <v>322.9</v>
+      </c>
       <c r="Z61" s="8" t="n">
         <v>0.13</v>
       </c>
@@ -7612,7 +7638,7 @@
       </c>
       <c r="AX61" s="8" t="inlineStr">
         <is>
-          <t>N.S.I. = Non-Schedule Item (rate outside DSR 1989); Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - concrete, 30-35 MPa, general mix</t>
+          <t>N.S.I. = Non-Schedule Item (rate outside DSR 1989); Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - concrete, 30-35 MPa, general mix; Mass derived from length x 22500.0 sq.mm cross-section (from BoQ description) x density; Gola cross-section treated as full 15x15cm square; actual filleted profile is smaller, so mass is an upper-bound estimate</t>
         </is>
       </c>
     </row>
@@ -7687,7 +7713,9 @@
       <c r="X62" s="8" t="n">
         <v>2400</v>
       </c>
-      <c r="Y62" s="8" t="n"/>
+      <c r="Y62" s="8" t="n">
+        <v>9.5</v>
+      </c>
       <c r="Z62" s="8" t="n">
         <v>0.13</v>
       </c>
@@ -7728,7 +7756,7 @@
       </c>
       <c r="AX62" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - concrete, 30-35 MPa, general mix</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - concrete, 30-35 MPa, general mix; Mass derived from count x 10125.0 cu.cm volume per unit (from BoQ description) x density</t>
         </is>
       </c>
     </row>
@@ -8359,7 +8387,9 @@
       <c r="X68" s="8" t="n">
         <v>1900</v>
       </c>
-      <c r="Y68" s="8" t="n"/>
+      <c r="Y68" s="8" t="n">
+        <v>787.5</v>
+      </c>
       <c r="Z68" s="8" t="n">
         <v>0.157</v>
       </c>
@@ -8400,7 +8430,7 @@
       </c>
       <c r="AX68" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - mortar (1:6 cement:sand, general)</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - mortar (1:6 cement:sand, general); Mass derived from area x 12mm thickness (from BoQ description) x density</t>
         </is>
       </c>
     </row>
@@ -8483,7 +8513,9 @@
       <c r="X69" s="8" t="n">
         <v>1900</v>
       </c>
-      <c r="Y69" s="8" t="n"/>
+      <c r="Y69" s="8" t="n">
+        <v>984.4</v>
+      </c>
       <c r="Z69" s="8" t="n">
         <v>0.157</v>
       </c>
@@ -8524,7 +8556,7 @@
       </c>
       <c r="AX69" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - mortar (1:6 cement:sand, general)</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - mortar (1:6 cement:sand, general); Mass derived from area x 15mm thickness (from BoQ description) x density</t>
         </is>
       </c>
     </row>
@@ -8607,7 +8639,9 @@
       <c r="X70" s="8" t="n">
         <v>1900</v>
       </c>
-      <c r="Y70" s="8" t="n"/>
+      <c r="Y70" s="8" t="n">
+        <v>34</v>
+      </c>
       <c r="Z70" s="8" t="n">
         <v>0.157</v>
       </c>
@@ -8648,7 +8682,7 @@
       </c>
       <c r="AX70" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - mortar (1:6 cement:sand, general)</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - mortar (1:6 cement:sand, general); Mass derived from area x 6mm thickness (from BoQ description) x density</t>
         </is>
       </c>
     </row>
@@ -8731,7 +8765,9 @@
       <c r="X71" s="8" t="n">
         <v>2700</v>
       </c>
-      <c r="Y71" s="8" t="n"/>
+      <c r="Y71" s="8" t="n">
+        <v>76.8</v>
+      </c>
       <c r="Z71" s="8" t="n">
         <v>0.079</v>
       </c>
@@ -8772,7 +8808,7 @@
       </c>
       <c r="AX71" s="8" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - marble/dimension stone</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - marble/dimension stone; Mass derived from area x 18mm thickness (from BoQ description) x density; Composite assembly: mass uses only the top finish layer's stated thickness/density; underlayer(s) of a different material are excluded</t>
         </is>
       </c>
     </row>
@@ -9636,6 +9672,9 @@
       <c r="X80" t="n">
         <v>2400</v>
       </c>
+      <c r="Y80" t="n">
+        <v>539.8</v>
+      </c>
       <c r="Z80" t="n">
         <v>0.13</v>
       </c>
@@ -9664,7 +9703,7 @@
       </c>
       <c r="AX80" t="inlineStr">
         <is>
-          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - concrete, 30-35 MPa, general mix</t>
+          <t>Embodied carbon source: ICE Database v3.0 (Circular Ecology, Univ. of Bath, 2019) - concrete, 30-35 MPa, general mix; Mass derived from area x 50mm thickness (from BoQ description) x density</t>
         </is>
       </c>
     </row>

</xml_diff>